<commit_message>
feat: add LOC DMN rules, Docker/Quarkus setup, and Python test runner
- LOCCalculation.dmn: cascade flow (Limpieza → Calculos → LOC Result)
- Dockerfile: multi-stage build (Maven + JRE 17)
- pom.xml: Quarkus + Kogito dependencies
- run_test.py: build/start/test/stop automation
- Project structure: 02 Test, 03 Input, 04 Output
</commit_message>
<xml_diff>
--- a/00 Archivos/MetodologiaCalculo.xlsx
+++ b/00 Archivos/MetodologiaCalculo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericchirum/Library/Mobile Documents/com~apple~CloudDocs/10 Pro/01 LOC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericchirum/Library/Mobile Documents/com~apple~CloudDocs/10 Pro/01 LOC/00 Archivos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19C7AA5C-FA7A-014F-A99A-C4BB251D712E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3514D039-3383-924D-ACFC-04ABE3F28AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" activeTab="1" xr2:uid="{556D8836-4F9B-4CE7-9DBB-35AB4DE76F51}"/>
   </bookViews>

</xml_diff>